<commit_message>
Work Plan (4th Month)
</commit_message>
<xml_diff>
--- a/4th month plan.xlsx
+++ b/4th month plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Daily-GitHub\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE66E2FB-0460-4E95-B5C0-609F0CC87E2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39FAEAC8-08BA-4085-9F4D-562F3753823F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{EF880F71-DA17-459F-94A4-8E740AADF52E}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="63">
   <si>
     <t>Day</t>
   </si>
@@ -42,60 +42,21 @@
     <t>Platform / Task Type</t>
   </si>
   <si>
-    <t>Task / Problem</t>
-  </si>
-  <si>
     <t>Concept Focus</t>
   </si>
   <si>
     <t>LeetCode</t>
   </si>
   <si>
-    <t>Implement Stack using Array (#225, Easy)</t>
-  </si>
-  <si>
-    <t>Stack, Array Implementation</t>
-  </si>
-  <si>
     <t>HackerRank</t>
   </si>
   <si>
-    <t>Implement Queue using Linked List</t>
-  </si>
-  <si>
-    <t>Queue, Linked List</t>
-  </si>
-  <si>
     <t>GeeksforGeeks</t>
   </si>
   <si>
-    <t>Create Class with Constructor, Destructor, and Member Functions</t>
-  </si>
-  <si>
-    <t>OOPs Basics, Constructor/Destructor</t>
-  </si>
-  <si>
     <t>Pandas / NumPy / SQL</t>
   </si>
   <si>
-    <t>Bar chart of monthly sales from CSV</t>
-  </si>
-  <si>
-    <t>Data Visualization, CSV Handling</t>
-  </si>
-  <si>
-    <t>Binary Search (Recursive &amp; Iterative) (#704, Easy)</t>
-  </si>
-  <si>
-    <t>Searching, Recursion</t>
-  </si>
-  <si>
-    <t>Pointer arithmetic and array manipulation</t>
-  </si>
-  <si>
-    <t>Pointers, Array Access</t>
-  </si>
-  <si>
     <t>Free / Revision Day</t>
   </si>
   <si>
@@ -105,140 +66,170 @@
     <t>Review Days 91–96 or rest</t>
   </si>
   <si>
-    <t>Implement Linked List operations (Insert, Delete)</t>
-  </si>
-  <si>
-    <t>Linked List, Dynamic Memory</t>
-  </si>
-  <si>
-    <t>Read/Write text files (simulate using #file I/O problems)</t>
-  </si>
-  <si>
-    <t>File Handling Basics</t>
-  </si>
-  <si>
-    <t>Line chart of stock prices from CSV</t>
-  </si>
-  <si>
-    <t>Data Visualization, Pandas</t>
-  </si>
-  <si>
-    <t>Reverse a Linked List (#206, Easy)</t>
-  </si>
-  <si>
-    <t>Linked List Manipulation</t>
-  </si>
-  <si>
-    <t>Merge Two Sorted Linked Lists (#21, Easy)</t>
-  </si>
-  <si>
-    <t>Linked List, Two-pointer Technique</t>
-  </si>
-  <si>
-    <t>Inheritance: Base and Derived class, method overriding (#133, Easy for OO simulation)</t>
-  </si>
-  <si>
-    <t>Inheritance, Polymorphism</t>
-  </si>
-  <si>
     <t>Review Days 98–103 or backlog</t>
   </si>
   <si>
-    <t>Implement Queue using Two Stacks</t>
-  </si>
-  <si>
-    <t>Stack, Queue Simulation</t>
-  </si>
-  <si>
-    <t>Dynamic Memory Allocation (new/delete)</t>
-  </si>
-  <si>
-    <t>Pointers, Memory Management</t>
-  </si>
-  <si>
-    <t>Detect Loop in Linked List (#141, Easy)</t>
-  </si>
-  <si>
-    <t>Linked List, Cycle Detection</t>
-  </si>
-  <si>
-    <t>Pivot table: Total sales by region and product</t>
-  </si>
-  <si>
-    <t>Aggregation, Pandas</t>
-  </si>
-  <si>
-    <t>Copy contents of one file to another file</t>
-  </si>
-  <si>
-    <t>File Streams, I/O</t>
-  </si>
-  <si>
-    <t>Implement Stack using Linked List</t>
-  </si>
-  <si>
     <t>Stack, Linked List</t>
   </si>
   <si>
     <t>Review Days 105–110 or rest</t>
   </si>
   <si>
-    <t>Implement Queue using Circular Array (#622, Medium)</t>
-  </si>
-  <si>
-    <t>Queue, Array Implementation</t>
-  </si>
-  <si>
-    <t>Abstract class and Pure Virtual Function</t>
-  </si>
-  <si>
-    <t>OOPs, Abstraction</t>
-  </si>
-  <si>
-    <t>Implement Priority Queue using Array</t>
-  </si>
-  <si>
-    <t>Heap, Array</t>
-  </si>
-  <si>
-    <t>Pointer to Pointer &amp; Dynamic 2D Array (#59, Medium for 2D DP)</t>
-  </si>
-  <si>
-    <t>Advanced Pointers, 2D Memory</t>
-  </si>
-  <si>
     <t>SQL: Find employees with salary above average</t>
   </si>
   <si>
-    <t>SQL, Aggregation</t>
-  </si>
-  <si>
-    <t>Binary Tree: Insert &amp; Inorder Traversal</t>
-  </si>
-  <si>
-    <t>Trees, Recursion</t>
-  </si>
-  <si>
     <t>Review Days 112–117 or backlog</t>
   </si>
   <si>
-    <t>Implement Hash Table using Chaining</t>
-  </si>
-  <si>
-    <t>Hashing, Collision Handling</t>
-  </si>
-  <si>
-    <t>Dynamic Programming: Fibonacci using Memoization (#509, Easy)</t>
-  </si>
-  <si>
-    <t>DP, Recursion</t>
+    <t>Task / Problem (search / click to open)</t>
+  </si>
+  <si>
+    <t>Implement Stack using Queues (#225, Easy)</t>
+  </si>
+  <si>
+    <t>Stack Implementation</t>
+  </si>
+  <si>
+    <t>Queue using Two Stacks — https://www.hackerrank.com/challenges/queue-using-two-stacks/problem</t>
+  </si>
+  <si>
+    <t>Queue Logic</t>
+  </si>
+  <si>
+    <t>Geek and Coffee Shop — https://practice.geeksforgeeks.org/problems/geek-and-coffee-shop/0</t>
+  </si>
+  <si>
+    <t>OOPs, Constructor/Destructor</t>
+  </si>
+  <si>
+    <t>Pandas: Create bar chart from monthly sales CSV</t>
+  </si>
+  <si>
+    <t>Data Visualization</t>
+  </si>
+  <si>
+    <t>Binary Search (#704, Easy)</t>
+  </si>
+  <si>
+    <t>Searching</t>
+  </si>
+  <si>
+    <t>Pointers in C — https://www.hackerrank.com/challenges/pointer-in-c/problem</t>
+  </si>
+  <si>
+    <t>Pointer arithmetic, memory</t>
+  </si>
+  <si>
+    <t>Linked List Insertion — https://practice.geeksforgeeks.org/problems/linked-list-insertion/1</t>
+  </si>
+  <si>
+    <t>Linked List</t>
+  </si>
+  <si>
+    <t>Reverse String (#344, Easy)</t>
+  </si>
+  <si>
+    <t>String Manipulation</t>
+  </si>
+  <si>
+    <t>Pandas: Line Chart of Stock Prices from CSV</t>
+  </si>
+  <si>
+    <t>Reverse a Linked List — https://www.hackerrank.com/challenges/reverse-a-linked-list/problem</t>
+  </si>
+  <si>
+    <t>Merge Two Sorted Linked Lists — https://practice.geeksforgeeks.org/problems/merge-two-sorted-linked-lists/1</t>
+  </si>
+  <si>
+    <t>Linked List, Two-pointers</t>
+  </si>
+  <si>
+    <t>Clone Graph (#133, Medium)</t>
+  </si>
+  <si>
+    <t>Graph, OOP-like structure</t>
+  </si>
+  <si>
+    <t>Stack / Queue simulation</t>
+  </si>
+  <si>
+    <t>Dynamic Memory Allocation (practice) — https://practice.geeksforgeeks.org/problems/dynamic-memory-allocation/1</t>
+  </si>
+  <si>
+    <t>new/delete, memory mgmt</t>
+  </si>
+  <si>
+    <t>Linked List Cycle (#141, Easy)</t>
+  </si>
+  <si>
+    <t>Cycle Detection</t>
+  </si>
+  <si>
+    <t>Pandas: Create Pivot Table (Sales by Region × Product)</t>
+  </si>
+  <si>
+    <t>Aggregation</t>
+  </si>
+  <si>
+    <t>StringStream — https://www.hackerrank.com/challenges/c-tutorial-stringstream/problem</t>
+  </si>
+  <si>
+    <t>stringstream / parsing (I/O)</t>
+  </si>
+  <si>
+    <t>Implement Stack Using Linked List — https://practice.geeksforgeeks.org/problems/implement-stack-using-linked-list/1</t>
+  </si>
+  <si>
+    <t>Design Circular Queue (#622, Medium)</t>
+  </si>
+  <si>
+    <t>Circular Queue design</t>
+  </si>
+  <si>
+    <t>Abstract Classes - Polymorphism — https://www.hackerrank.com/challenges/abstract-classes-polymorphism/problem</t>
+  </si>
+  <si>
+    <t>OOP, Abstraction</t>
+  </si>
+  <si>
+    <t>Implementation of Priority Queue using Binary Heap — https://practice.geeksforgeeks.org/problems/implementation-of-priority-queue-using-binary-heap/1</t>
+  </si>
+  <si>
+    <t>Priority Queue (heap)</t>
+  </si>
+  <si>
+    <t>Spiral Matrix II (#59, Medium)</t>
+  </si>
+  <si>
+    <t>2D arrays, index math</t>
+  </si>
+  <si>
+    <t>SQL aggregation</t>
+  </si>
+  <si>
+    <t>Binary Search Tree: Insertion — https://www.hackerrank.com/challenges/binary-search-tree-insertion/problem</t>
+  </si>
+  <si>
+    <t>Trees</t>
+  </si>
+  <si>
+    <t>Separate Chaining in Hashing (practice) — https://practice.geeksforgeeks.org/problems/separate-chaining-in-hashing-1587115621--124916/1</t>
+  </si>
+  <si>
+    <t>Hashing, collision handling</t>
+  </si>
+  <si>
+    <t>Fibonacci Number (#509, Easy)</t>
+  </si>
+  <si>
+    <t>Dynamic Programming, Memoization</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -250,6 +241,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -272,10 +271,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -286,8 +286,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -608,7 +612,7 @@
     <col min="4" max="4" width="29.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -616,433 +620,449 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:4" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>91</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="64.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>92</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>8</v>
+      <c r="B3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>18</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="62.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>93</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>11</v>
+      <c r="B4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>20</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>94</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>14</v>
+      <c r="B5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>95</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>16</v>
+      <c r="B6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>24</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>96</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>18</v>
+      <c r="B7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>26</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>97</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>20</v>
+      <c r="B8" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>98</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>23</v>
+      <c r="B9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>28</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>99</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>25</v>
+      <c r="B10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>30</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>100</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>27</v>
+      <c r="B11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>32</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="63.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>101</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="B12" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:4" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>102</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>31</v>
+      <c r="B13" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>34</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>103</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>33</v>
+      <c r="B14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>36</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>104</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>20</v>
+      <c r="B15" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="62.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>105</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>36</v>
+      <c r="B16" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>18</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>106</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>38</v>
+      <c r="B17" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>39</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>107</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>40</v>
+      <c r="B18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>108</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>42</v>
+      <c r="B19" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>43</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="67.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>109</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>44</v>
+      <c r="B20" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>45</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="81" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>110</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>46</v>
+      <c r="B21" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>47</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>47</v>
+        <v>11</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>111</v>
       </c>
-      <c r="B22" s="3" t="s">
-        <v>20</v>
+      <c r="B22" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>112</v>
       </c>
-      <c r="B23" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C23" s="2" t="s">
+      <c r="B23" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:4" ht="78.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>113</v>
       </c>
-      <c r="B24" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C24" s="2" t="s">
+      <c r="B24" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:4" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>114</v>
       </c>
-      <c r="B25" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C25" s="2" t="s">
+      <c r="B25" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:4" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>115</v>
       </c>
-      <c r="B26" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C26" s="2" t="s">
+      <c r="B26" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>116</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C27" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="D27" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="63.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>117</v>
       </c>
-      <c r="B28" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>59</v>
+      <c r="B28" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>57</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>118</v>
       </c>
-      <c r="B29" s="3" t="s">
-        <v>20</v>
+      <c r="B29" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="73.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>119</v>
       </c>
-      <c r="B30" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>62</v>
+      <c r="B30" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>59</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>120</v>
       </c>
-      <c r="B31" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>64</v>
+      <c r="B31" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C3" r:id="rId1" display="https://www.hackerrank.com/challenges/queue-using-two-stacks/problem" xr:uid="{B309DE2C-FC4D-438F-9CBB-6E86BD2CA85C}"/>
+    <hyperlink ref="C4" r:id="rId2" display="https://practice.geeksforgeeks.org/problems/geek-and-coffee-shop/0" xr:uid="{003C2D06-5D36-4379-8C91-E2C1F55990F4}"/>
+    <hyperlink ref="C7" r:id="rId3" display="https://www.hackerrank.com/challenges/pointer-in-c/problem" xr:uid="{B4FDDDC4-6DB6-44F0-ACEF-9F61457A0508}"/>
+    <hyperlink ref="C9" r:id="rId4" display="https://practice.geeksforgeeks.org/problems/linked-list-insertion/1" xr:uid="{CC9FDA3B-F4FB-4C85-8497-22FFD305E1B6}"/>
+    <hyperlink ref="C12" r:id="rId5" display="https://www.hackerrank.com/challenges/reverse-a-linked-list/problem" xr:uid="{D7342DFE-B534-41A2-BC39-A3300BA46235}"/>
+    <hyperlink ref="C13" r:id="rId6" display="https://practice.geeksforgeeks.org/problems/merge-two-sorted-linked-lists/1" xr:uid="{CAAA3591-E64A-4CE4-BBB1-1BCE879231D4}"/>
+    <hyperlink ref="C16" r:id="rId7" display="https://www.hackerrank.com/challenges/queue-using-two-stacks/problem" xr:uid="{0C4B7882-02BA-45DF-96CB-6FF426399794}"/>
+    <hyperlink ref="C17" r:id="rId8" display="https://practice.geeksforgeeks.org/problems/dynamic-memory-allocation/1" xr:uid="{796DFB61-067B-4753-8959-3DE598628BF6}"/>
+    <hyperlink ref="C20" r:id="rId9" display="https://www.hackerrank.com/challenges/c-tutorial-stringstream/problem" xr:uid="{9BE1D1B4-4DAE-42EC-BDA6-1844786FAD54}"/>
+    <hyperlink ref="C21" r:id="rId10" display="https://practice.geeksforgeeks.org/problems/implement-stack-using-linked-list/1" xr:uid="{3B2C593C-BF41-4043-BDDB-8CCFB549021E}"/>
+    <hyperlink ref="C24" r:id="rId11" display="https://www.hackerrank.com/challenges/abstract-classes-polymorphism/problem" xr:uid="{6B026FE4-33E5-42E4-A5FF-C0DACC27C46C}"/>
+    <hyperlink ref="C25" r:id="rId12" display="https://practice.geeksforgeeks.org/problems/implementation-of-priority-queue-using-binary-heap/1" xr:uid="{932EA6ED-C0C7-4257-A772-6B7E6269DABA}"/>
+    <hyperlink ref="C28" r:id="rId13" display="https://www.hackerrank.com/challenges/binary-search-tree-insertion/problem" xr:uid="{66CE15EF-47F9-4C9B-BEC8-97E240F2478F}"/>
+    <hyperlink ref="C30" r:id="rId14" display="https://practice.geeksforgeeks.org/problems/separate-chaining-in-hashing-1587115621--124916/1" xr:uid="{E169D0FC-33ED-4842-AC65-408AD1833AAF}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>